<commit_message>
Updated NGA_grids_kan10 model - 2026-06-18 23:34
</commit_message>
<xml_diff>
--- a/VerveStacks_NGA_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NGA_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NGA_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{17B2B8C7-E741-49DE-93BA-D0329A875EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A337A1F-F647-474A-A86E-632A7A4584AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19530,7 +19530,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90A380F-0D68-4326-86F1-8E4E1463910C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A343581D-4B02-4014-AD78-8F1977A11FDF}">
   <dimension ref="B9:H98"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21328,7 +21328,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9BC1D9B-AF3C-4173-8CDA-952E4A6F1D2B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00C7DC65-F985-4A76-8DD5-E7C3DD884950}">
   <dimension ref="B9:L98"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>